<commit_message>
latest update for may 2026 class
</commit_message>
<xml_diff>
--- a/lab stuff/regression/Predictive-Maintenance-pt1.xlsx
+++ b/lab stuff/regression/Predictive-Maintenance-pt1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\workshops\data science\intro keysight\main labs\regression\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\temp\intro data science labs\regression\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1005BA2E-80A3-47B2-AD89-E516BE4DB09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E484BFC0-E979-485D-B9A8-3EEC930DB85B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Initial" sheetId="6" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="34">
   <si>
     <t>Coefficients</t>
   </si>
@@ -131,12 +131,21 @@
   <si>
     <t>Air temperature</t>
   </si>
+  <si>
+    <t>Variables to be included: Humidity, Rotational Speed, Downtime (Hours)</t>
+  </si>
+  <si>
+    <t>Variables to be excluded: Noise Level</t>
+  </si>
+  <si>
+    <t>Variables to be excluded: Noise Level, Air Temperature</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -160,13 +169,51 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -201,11 +248,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -214,9 +272,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,40 +565,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC29C866-C764-4D56-9889-FCA9CE139B86}">
   <dimension ref="B2:H42"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.265625" customWidth="1"/>
-    <col min="3" max="3" width="11.9296875" customWidth="1"/>
-    <col min="4" max="4" width="10.53125" customWidth="1"/>
-    <col min="5" max="6" width="12.9296875" customWidth="1"/>
-    <col min="7" max="7" width="13.265625" customWidth="1"/>
-    <col min="8" max="8" width="15.265625" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" customWidth="1"/>
+    <col min="6" max="6" width="13.21875" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" ht="47.25" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:8" ht="31.2" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="19" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>1</v>
       </c>
@@ -545,16 +613,16 @@
         <v>20</v>
       </c>
       <c r="F3">
+        <v>59</v>
+      </c>
+      <c r="G3">
         <v>6</v>
       </c>
-      <c r="G3">
-        <v>34</v>
-      </c>
-      <c r="H3">
+      <c r="H3" s="20">
         <v>-40.199999999999989</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>2</v>
       </c>
@@ -568,16 +636,16 @@
         <v>12</v>
       </c>
       <c r="F4">
+        <v>-38</v>
+      </c>
+      <c r="G4">
         <v>20</v>
       </c>
-      <c r="G4">
-        <v>15</v>
-      </c>
-      <c r="H4">
+      <c r="H4" s="20">
         <v>57.399999999999977</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>3</v>
       </c>
@@ -591,16 +659,16 @@
         <v>16</v>
       </c>
       <c r="F5">
+        <v>15</v>
+      </c>
+      <c r="G5">
         <v>16</v>
       </c>
-      <c r="G5">
-        <v>46</v>
-      </c>
-      <c r="H5">
+      <c r="H5" s="20">
         <v>-139.39999999999998</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>4</v>
       </c>
@@ -614,16 +682,16 @@
         <v>42</v>
       </c>
       <c r="F6">
+        <v>-16</v>
+      </c>
+      <c r="G6">
         <v>13</v>
       </c>
-      <c r="G6">
-        <v>15</v>
-      </c>
-      <c r="H6">
+      <c r="H6" s="20">
         <v>-55.200000000000017</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>5</v>
       </c>
@@ -637,16 +705,16 @@
         <v>43</v>
       </c>
       <c r="F7">
+        <v>78</v>
+      </c>
+      <c r="G7">
         <v>9</v>
       </c>
-      <c r="G7">
-        <v>-14</v>
-      </c>
-      <c r="H7">
+      <c r="H7" s="20">
         <v>11.299999999999955</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>6</v>
       </c>
@@ -660,16 +728,16 @@
         <v>47</v>
       </c>
       <c r="F8">
+        <v>-22</v>
+      </c>
+      <c r="G8">
         <v>13</v>
       </c>
-      <c r="G8">
-        <v>65</v>
-      </c>
-      <c r="H8">
+      <c r="H8" s="20">
         <v>187.9</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>7</v>
       </c>
@@ -683,16 +751,16 @@
         <v>20</v>
       </c>
       <c r="F9">
+        <v>-79</v>
+      </c>
+      <c r="G9">
         <v>14</v>
       </c>
-      <c r="G9">
-        <v>3</v>
-      </c>
-      <c r="H9">
+      <c r="H9" s="20">
         <v>-171.6</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>8</v>
       </c>
@@ -706,16 +774,16 @@
         <v>39</v>
       </c>
       <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10">
         <v>9</v>
       </c>
-      <c r="G10">
-        <v>38</v>
-      </c>
-      <c r="H10">
+      <c r="H10" s="20">
         <v>-88.90000000000002</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>9</v>
       </c>
@@ -729,16 +797,16 @@
         <v>29</v>
       </c>
       <c r="F11">
+        <v>-43</v>
+      </c>
+      <c r="G11">
         <v>15</v>
       </c>
-      <c r="G11">
-        <v>47</v>
-      </c>
-      <c r="H11">
+      <c r="H11" s="20">
         <v>-54.700000000000045</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>10</v>
       </c>
@@ -752,16 +820,16 @@
         <v>46</v>
       </c>
       <c r="F12">
+        <v>74</v>
+      </c>
+      <c r="G12">
         <v>3</v>
       </c>
-      <c r="G12">
-        <v>2</v>
-      </c>
-      <c r="H12">
+      <c r="H12" s="20">
         <v>48.400000000000006</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>11</v>
       </c>
@@ -775,16 +843,16 @@
         <v>48</v>
       </c>
       <c r="F13">
+        <v>-59</v>
+      </c>
+      <c r="G13">
         <v>7</v>
       </c>
-      <c r="G13">
-        <v>-2</v>
-      </c>
-      <c r="H13">
+      <c r="H13" s="20">
         <v>-10.400000000000034</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14">
         <v>12</v>
       </c>
@@ -798,16 +866,16 @@
         <v>26</v>
       </c>
       <c r="F14">
+        <v>-46</v>
+      </c>
+      <c r="G14">
         <v>6</v>
       </c>
-      <c r="G14">
-        <v>75</v>
-      </c>
-      <c r="H14">
+      <c r="H14" s="20">
         <v>-58.200000000000017</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>13</v>
       </c>
@@ -821,16 +889,16 @@
         <v>36</v>
       </c>
       <c r="F15">
+        <v>-37</v>
+      </c>
+      <c r="G15">
         <v>21</v>
       </c>
-      <c r="G15">
-        <v>80</v>
-      </c>
-      <c r="H15">
+      <c r="H15" s="20">
         <v>-7.2000000000000171</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16">
         <v>14</v>
       </c>
@@ -844,16 +912,16 @@
         <v>46</v>
       </c>
       <c r="F16">
+        <v>-18</v>
+      </c>
+      <c r="G16">
         <v>6</v>
       </c>
-      <c r="G16">
-        <v>86</v>
-      </c>
-      <c r="H16">
+      <c r="H16" s="20">
         <v>54.800000000000011</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>15</v>
       </c>
@@ -867,16 +935,16 @@
         <v>29</v>
       </c>
       <c r="F17">
+        <v>-52</v>
+      </c>
+      <c r="G17">
         <v>7</v>
       </c>
-      <c r="G17">
-        <v>35</v>
-      </c>
-      <c r="H17">
+      <c r="H17" s="20">
         <v>-68.100000000000009</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>16</v>
       </c>
@@ -890,16 +958,16 @@
         <v>11</v>
       </c>
       <c r="F18">
+        <v>16</v>
+      </c>
+      <c r="G18">
         <v>17</v>
       </c>
-      <c r="G18">
-        <v>37</v>
-      </c>
-      <c r="H18">
+      <c r="H18" s="20">
         <v>-65.09999999999998</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>17</v>
       </c>
@@ -913,16 +981,16 @@
         <v>30</v>
       </c>
       <c r="F19">
+        <v>-34</v>
+      </c>
+      <c r="G19">
         <v>19</v>
       </c>
-      <c r="G19">
-        <v>59</v>
-      </c>
-      <c r="H19">
+      <c r="H19" s="20">
         <v>78.800000000000011</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>18</v>
       </c>
@@ -936,16 +1004,16 @@
         <v>32</v>
       </c>
       <c r="F20">
+        <v>63</v>
+      </c>
+      <c r="G20">
         <v>14</v>
       </c>
-      <c r="G20">
-        <v>84</v>
-      </c>
-      <c r="H20">
+      <c r="H20" s="20">
         <v>-120.19999999999999</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>19</v>
       </c>
@@ -959,16 +1027,16 @@
         <v>34</v>
       </c>
       <c r="F21">
+        <v>76</v>
+      </c>
+      <c r="G21">
         <v>7</v>
       </c>
-      <c r="G21">
-        <v>9</v>
-      </c>
-      <c r="H21">
+      <c r="H21" s="20">
         <v>-48.000000000000014</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>20</v>
       </c>
@@ -982,16 +1050,16 @@
         <v>45</v>
       </c>
       <c r="F22">
+        <v>-29</v>
+      </c>
+      <c r="G22">
         <v>17</v>
       </c>
-      <c r="G22">
-        <v>55</v>
-      </c>
-      <c r="H22">
+      <c r="H22" s="20">
         <v>262.10000000000002</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>21</v>
       </c>
@@ -1005,16 +1073,16 @@
         <v>17</v>
       </c>
       <c r="F23">
+        <v>43</v>
+      </c>
+      <c r="G23">
         <v>10</v>
       </c>
-      <c r="G23">
-        <v>50</v>
-      </c>
-      <c r="H23">
+      <c r="H23" s="20">
         <v>-153.70000000000002</v>
       </c>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B24">
         <v>22</v>
       </c>
@@ -1028,16 +1096,16 @@
         <v>15</v>
       </c>
       <c r="F24">
+        <v>-19</v>
+      </c>
+      <c r="G24">
         <v>14</v>
       </c>
-      <c r="G24">
-        <v>-3</v>
-      </c>
-      <c r="H24">
+      <c r="H24" s="20">
         <v>-65.099999999999994</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B25">
         <v>23</v>
       </c>
@@ -1051,16 +1119,16 @@
         <v>24</v>
       </c>
       <c r="F25">
+        <v>-60</v>
+      </c>
+      <c r="G25">
         <v>2</v>
       </c>
-      <c r="G25">
-        <v>-14</v>
-      </c>
-      <c r="H25">
+      <c r="H25" s="20">
         <v>-190.60000000000002</v>
       </c>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B26">
         <v>24</v>
       </c>
@@ -1074,16 +1142,16 @@
         <v>22</v>
       </c>
       <c r="F26">
+        <v>-20</v>
+      </c>
+      <c r="G26">
         <v>9</v>
       </c>
-      <c r="G26">
-        <v>71</v>
-      </c>
-      <c r="H26">
+      <c r="H26" s="20">
         <v>0.80000000000001137</v>
       </c>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B27">
         <v>25</v>
       </c>
@@ -1097,16 +1165,16 @@
         <v>23</v>
       </c>
       <c r="F27">
+        <v>-70</v>
+      </c>
+      <c r="G27">
         <v>23</v>
       </c>
-      <c r="G27">
-        <v>32</v>
-      </c>
-      <c r="H27">
+      <c r="H27" s="20">
         <v>154.69999999999999</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B28">
         <v>26</v>
       </c>
@@ -1120,16 +1188,16 @@
         <v>46</v>
       </c>
       <c r="F28">
+        <v>-83</v>
+      </c>
+      <c r="G28">
         <v>10</v>
       </c>
-      <c r="G28">
-        <v>-20</v>
-      </c>
-      <c r="H28">
+      <c r="H28" s="20">
         <v>-19</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B29">
         <v>27</v>
       </c>
@@ -1143,16 +1211,16 @@
         <v>44</v>
       </c>
       <c r="F29">
+        <v>95</v>
+      </c>
+      <c r="G29">
         <v>18</v>
       </c>
-      <c r="G29">
-        <v>38</v>
-      </c>
-      <c r="H29">
+      <c r="H29" s="20">
         <v>57.599999999999994</v>
       </c>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B30">
         <v>28</v>
       </c>
@@ -1166,16 +1234,16 @@
         <v>23</v>
       </c>
       <c r="F30">
+        <v>-24</v>
+      </c>
+      <c r="G30">
         <v>9</v>
       </c>
-      <c r="G30">
-        <v>75</v>
-      </c>
-      <c r="H30">
+      <c r="H30" s="20">
         <v>-145.89999999999998</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B31">
         <v>29</v>
       </c>
@@ -1189,16 +1257,16 @@
         <v>25</v>
       </c>
       <c r="F31">
+        <v>28</v>
+      </c>
+      <c r="G31">
         <v>2</v>
       </c>
-      <c r="G31">
-        <v>42</v>
-      </c>
-      <c r="H31">
+      <c r="H31" s="20">
         <v>-147.50000000000003</v>
       </c>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B32">
         <v>30</v>
       </c>
@@ -1212,16 +1280,16 @@
         <v>44</v>
       </c>
       <c r="F32">
+        <v>60</v>
+      </c>
+      <c r="G32">
         <v>21</v>
       </c>
-      <c r="G32">
-        <v>25</v>
-      </c>
-      <c r="H32">
+      <c r="H32" s="20">
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B33">
         <v>31</v>
       </c>
@@ -1235,16 +1303,16 @@
         <v>48</v>
       </c>
       <c r="F33">
+        <v>-4</v>
+      </c>
+      <c r="G33">
         <v>12</v>
       </c>
-      <c r="G33">
-        <v>70</v>
-      </c>
-      <c r="H33">
+      <c r="H33" s="20">
         <v>177.60000000000002</v>
       </c>
     </row>
-    <row r="34" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B34">
         <v>32</v>
       </c>
@@ -1258,16 +1326,16 @@
         <v>23</v>
       </c>
       <c r="F34">
+        <v>-73</v>
+      </c>
+      <c r="G34">
         <v>17</v>
       </c>
-      <c r="G34">
-        <v>8</v>
-      </c>
-      <c r="H34">
+      <c r="H34" s="20">
         <v>9.1000000000000227</v>
       </c>
     </row>
-    <row r="35" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B35">
         <v>33</v>
       </c>
@@ -1281,16 +1349,16 @@
         <v>19</v>
       </c>
       <c r="F35">
+        <v>-67</v>
+      </c>
+      <c r="G35">
         <v>15</v>
       </c>
-      <c r="G35">
-        <v>-8</v>
-      </c>
-      <c r="H35">
+      <c r="H35" s="20">
         <v>-42.5</v>
       </c>
     </row>
-    <row r="36" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B36">
         <v>34</v>
       </c>
@@ -1304,16 +1372,16 @@
         <v>10</v>
       </c>
       <c r="F36">
+        <v>-29</v>
+      </c>
+      <c r="G36">
         <v>8</v>
       </c>
-      <c r="G36">
-        <v>7</v>
-      </c>
-      <c r="H36">
+      <c r="H36" s="20">
         <v>-172.8</v>
       </c>
     </row>
-    <row r="37" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B37">
         <v>35</v>
       </c>
@@ -1327,16 +1395,16 @@
         <v>14</v>
       </c>
       <c r="F37">
+        <v>-37</v>
+      </c>
+      <c r="G37">
         <v>6</v>
       </c>
-      <c r="G37">
-        <v>82</v>
-      </c>
-      <c r="H37">
+      <c r="H37" s="20">
         <v>-123.59999999999998</v>
       </c>
     </row>
-    <row r="38" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B38">
         <v>36</v>
       </c>
@@ -1350,16 +1418,16 @@
         <v>48</v>
       </c>
       <c r="F38">
+        <v>20</v>
+      </c>
+      <c r="G38">
         <v>5</v>
       </c>
-      <c r="G38">
-        <v>-20</v>
-      </c>
-      <c r="H38">
+      <c r="H38" s="20">
         <v>28.799999999999983</v>
       </c>
     </row>
-    <row r="39" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B39">
         <v>37</v>
       </c>
@@ -1373,16 +1441,16 @@
         <v>39</v>
       </c>
       <c r="F39">
+        <v>-9</v>
+      </c>
+      <c r="G39">
         <v>24</v>
       </c>
-      <c r="G39">
-        <v>35</v>
-      </c>
-      <c r="H39">
+      <c r="H39" s="20">
         <v>62.5</v>
       </c>
     </row>
-    <row r="40" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B40">
         <v>38</v>
       </c>
@@ -1396,16 +1464,16 @@
         <v>41</v>
       </c>
       <c r="F40">
+        <v>43</v>
+      </c>
+      <c r="G40">
         <v>11</v>
       </c>
-      <c r="G40">
-        <v>81</v>
-      </c>
-      <c r="H40">
+      <c r="H40" s="20">
         <v>-29.899999999999977</v>
       </c>
     </row>
-    <row r="41" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B41">
         <v>39</v>
       </c>
@@ -1419,16 +1487,16 @@
         <v>17</v>
       </c>
       <c r="F41">
+        <v>-8</v>
+      </c>
+      <c r="G41">
         <v>24</v>
       </c>
-      <c r="G41">
-        <v>-4</v>
-      </c>
-      <c r="H41">
+      <c r="H41" s="20">
         <v>-113.49999999999997</v>
       </c>
     </row>
-    <row r="42" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B42">
         <v>40</v>
       </c>
@@ -1442,12 +1510,12 @@
         <v>46</v>
       </c>
       <c r="F42">
+        <v>83</v>
+      </c>
+      <c r="G42">
         <v>9</v>
       </c>
-      <c r="G42">
-        <v>25</v>
-      </c>
-      <c r="H42">
+      <c r="H42" s="20">
         <v>82.399999999999977</v>
       </c>
     </row>
@@ -1458,18 +1526,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C07A71A2-9DED-4E4F-BA59-02680B5A1011}">
-  <dimension ref="B2:T51"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="B2:V73"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.3984375" customWidth="1"/>
-    <col min="3" max="3" width="13.06640625" customWidth="1"/>
-    <col min="4" max="4" width="15.265625" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="12.1328125" customWidth="1"/>
-    <col min="8" max="8" width="15.265625" customWidth="1"/>
+    <col min="6" max="6" width="11.21875" customWidth="1"/>
+    <col min="7" max="7" width="14.44140625" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+    <col min="12" max="12" width="25.77734375" customWidth="1"/>
+    <col min="13" max="13" width="11.44140625" customWidth="1"/>
+    <col min="16" max="16" width="23.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" ht="47.25" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:17" ht="46.8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
@@ -1482,17 +1554,17 @@
       <c r="E2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="19" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>1</v>
       </c>
@@ -1509,13 +1581,13 @@
         <v>42</v>
       </c>
       <c r="G3">
-        <v>34</v>
-      </c>
-      <c r="H3">
+        <v>59</v>
+      </c>
+      <c r="H3" s="20">
         <v>-40.199999999999989</v>
       </c>
     </row>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:17" ht="18" x14ac:dyDescent="0.35">
       <c r="B4">
         <v>2</v>
       </c>
@@ -1532,13 +1604,16 @@
         <v>30</v>
       </c>
       <c r="G4">
-        <v>15</v>
-      </c>
-      <c r="H4">
+        <v>-38</v>
+      </c>
+      <c r="H4" s="20">
         <v>57.399999999999977</v>
       </c>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.45">
+      <c r="L4" s="14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>3</v>
       </c>
@@ -1555,16 +1630,16 @@
         <v>23</v>
       </c>
       <c r="G5">
-        <v>46</v>
-      </c>
-      <c r="H5">
+        <v>15</v>
+      </c>
+      <c r="H5" s="20">
         <v>-139.39999999999998</v>
       </c>
       <c r="L5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>4</v>
       </c>
@@ -1581,13 +1656,13 @@
         <v>48</v>
       </c>
       <c r="G6">
-        <v>15</v>
-      </c>
-      <c r="H6">
+        <v>-16</v>
+      </c>
+      <c r="H6" s="20">
         <v>-55.200000000000017</v>
       </c>
     </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>5</v>
       </c>
@@ -1604,17 +1679,17 @@
         <v>42</v>
       </c>
       <c r="G7">
-        <v>-14</v>
-      </c>
-      <c r="H7">
+        <v>78</v>
+      </c>
+      <c r="H7" s="20">
         <v>11.299999999999955</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M7" s="5"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.45">
+      <c r="M7" s="4"/>
+    </row>
+    <row r="8" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>6</v>
       </c>
@@ -1631,19 +1706,19 @@
         <v>46</v>
       </c>
       <c r="G8">
-        <v>65</v>
-      </c>
-      <c r="H8">
+        <v>-22</v>
+      </c>
+      <c r="H8" s="20">
         <v>187.9</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" t="s">
         <v>3</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8">
         <v>0.96838085851750477</v>
       </c>
     </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>7</v>
       </c>
@@ -1660,19 +1735,19 @@
         <v>13</v>
       </c>
       <c r="G9">
-        <v>3</v>
-      </c>
-      <c r="H9">
+        <v>-79</v>
+      </c>
+      <c r="H9" s="20">
         <v>-171.6</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" t="s">
         <v>4</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9">
         <v>0.93776148714309959</v>
       </c>
     </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>8</v>
       </c>
@@ -1689,19 +1764,19 @@
         <v>50</v>
       </c>
       <c r="G10">
-        <v>38</v>
-      </c>
-      <c r="H10">
+        <v>4</v>
+      </c>
+      <c r="H10" s="20">
         <v>-88.90000000000002</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="12">
         <v>0.93257494440502464</v>
       </c>
     </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>9</v>
       </c>
@@ -1718,19 +1793,19 @@
         <v>46</v>
       </c>
       <c r="G11">
-        <v>47</v>
-      </c>
-      <c r="H11">
+        <v>-43</v>
+      </c>
+      <c r="H11" s="20">
         <v>-54.700000000000045</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" t="s">
         <v>6</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11">
         <v>27.694136134115027</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12">
         <v>10</v>
       </c>
@@ -1747,19 +1822,19 @@
         <v>33</v>
       </c>
       <c r="G12">
-        <v>2</v>
-      </c>
-      <c r="H12">
+        <v>74</v>
+      </c>
+      <c r="H12" s="20">
         <v>48.400000000000006</v>
       </c>
-      <c r="L12" s="3" t="s">
+      <c r="L12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="M12" s="3">
+      <c r="M12" s="2">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>11</v>
       </c>
@@ -1776,13 +1851,13 @@
         <v>33</v>
       </c>
       <c r="G13">
-        <v>-2</v>
-      </c>
-      <c r="H13">
+        <v>-59</v>
+      </c>
+      <c r="H13" s="20">
         <v>-10.400000000000034</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="2:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>12</v>
       </c>
@@ -1799,16 +1874,16 @@
         <v>20</v>
       </c>
       <c r="G14">
-        <v>75</v>
-      </c>
-      <c r="H14">
+        <v>-46</v>
+      </c>
+      <c r="H14" s="20">
         <v>-58.200000000000017</v>
       </c>
       <c r="L14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>13</v>
       </c>
@@ -1825,29 +1900,29 @@
         <v>24</v>
       </c>
       <c r="G15">
-        <v>80</v>
-      </c>
-      <c r="H15">
+        <v>-37</v>
+      </c>
+      <c r="H15" s="20">
         <v>-7.2000000000000171</v>
       </c>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4" t="s">
+      <c r="L15" s="3"/>
+      <c r="M15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="N15" s="4" t="s">
+      <c r="N15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O15" s="4" t="s">
+      <c r="O15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="P15" s="4" t="s">
+      <c r="P15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q15" s="4" t="s">
+      <c r="Q15" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B16">
         <v>14</v>
       </c>
@@ -1864,31 +1939,31 @@
         <v>16</v>
       </c>
       <c r="G16">
-        <v>86</v>
-      </c>
-      <c r="H16">
+        <v>-18</v>
+      </c>
+      <c r="H16" s="20">
         <v>54.800000000000011</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="L16" t="s">
         <v>9</v>
       </c>
-      <c r="M16" s="2">
+      <c r="M16">
         <v>3</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16">
         <v>416017.24340626388</v>
       </c>
-      <c r="O16" s="2">
+      <c r="O16">
         <v>138672.41446875464</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16">
         <v>180.80666341740147</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16">
         <v>9.3077244811578933E-22</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>15</v>
       </c>
@@ -1905,27 +1980,25 @@
         <v>44</v>
       </c>
       <c r="G17">
-        <v>35</v>
-      </c>
-      <c r="H17">
+        <v>-52</v>
+      </c>
+      <c r="H17" s="20">
         <v>-68.100000000000009</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="L17" t="s">
         <v>10</v>
       </c>
-      <c r="M17" s="2">
+      <c r="M17">
         <v>36</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17">
         <v>27610.746343736238</v>
       </c>
-      <c r="O17" s="2">
+      <c r="O17">
         <v>766.96517621489556</v>
       </c>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-    </row>
-    <row r="18" spans="2:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    </row>
+    <row r="18" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>16</v>
       </c>
@@ -1942,25 +2015,25 @@
         <v>45</v>
       </c>
       <c r="G18">
-        <v>37</v>
-      </c>
-      <c r="H18">
+        <v>16</v>
+      </c>
+      <c r="H18" s="20">
         <v>-65.09999999999998</v>
       </c>
-      <c r="L18" s="3" t="s">
+      <c r="L18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M18" s="3">
+      <c r="M18" s="2">
         <v>39</v>
       </c>
-      <c r="N18" s="3">
+      <c r="N18" s="2">
         <v>443627.98975000012</v>
       </c>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-    </row>
-    <row r="19" spans="2:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+    </row>
+    <row r="19" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>17</v>
       </c>
@@ -1977,13 +2050,13 @@
         <v>12</v>
       </c>
       <c r="G19">
-        <v>59</v>
-      </c>
-      <c r="H19">
+        <v>-34</v>
+      </c>
+      <c r="H19" s="20">
         <v>78.800000000000011</v>
       </c>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>18</v>
       </c>
@@ -2000,38 +2073,38 @@
         <v>17</v>
       </c>
       <c r="G20">
-        <v>84</v>
-      </c>
-      <c r="H20">
+        <v>63</v>
+      </c>
+      <c r="H20" s="20">
         <v>-120.19999999999999</v>
       </c>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4" t="s">
+      <c r="L20" s="3"/>
+      <c r="M20" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="N20" s="4" t="s">
+      <c r="N20" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="O20" s="4" t="s">
+      <c r="O20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="P20" s="4" t="s">
+      <c r="P20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Q20" s="4" t="s">
+      <c r="Q20" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="R20" s="4" t="s">
+      <c r="R20" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="S20" s="4" t="s">
+      <c r="S20" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="T20" s="4" t="s">
+      <c r="T20" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>19</v>
       </c>
@@ -2048,40 +2121,40 @@
         <v>48</v>
       </c>
       <c r="G21">
-        <v>9</v>
-      </c>
-      <c r="H21">
+        <v>76</v>
+      </c>
+      <c r="H21" s="20">
         <v>-48.000000000000014</v>
       </c>
-      <c r="L21" s="2" t="s">
+      <c r="L21" t="s">
         <v>12</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21">
         <v>-146.3321685353846</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21">
         <v>17.750570659780713</v>
       </c>
-      <c r="O21" s="2">
+      <c r="O21">
         <v>-8.2438007960467647</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21">
         <v>8.2612476509762775E-10</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21">
         <v>-182.33199440446549</v>
       </c>
-      <c r="R21" s="2">
+      <c r="R21">
         <v>-110.3323426663037</v>
       </c>
-      <c r="S21" s="2">
+      <c r="S21">
         <v>-182.33199440446549</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21">
         <v>-110.3323426663037</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>20</v>
       </c>
@@ -2098,40 +2171,40 @@
         <v>36</v>
       </c>
       <c r="G22">
-        <v>55</v>
-      </c>
-      <c r="H22">
+        <v>-29</v>
+      </c>
+      <c r="H22" s="20">
         <v>262.10000000000002</v>
       </c>
-      <c r="L22" s="2" t="s">
+      <c r="L22" t="s">
         <v>25</v>
       </c>
-      <c r="M22" s="2">
+      <c r="M22">
         <v>-3.4856110300186463</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22">
         <v>0.22669978631689819</v>
       </c>
-      <c r="O22" s="2">
+      <c r="O22">
         <v>-15.375449119948415</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22">
         <v>2.1350994941551336E-17</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22">
         <v>-3.9453795066714976</v>
       </c>
-      <c r="R22" s="2">
+      <c r="R22">
         <v>-3.0258425533657949</v>
       </c>
-      <c r="S22" s="2">
+      <c r="S22">
         <v>-3.9453795066714976</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22">
         <v>-3.0258425533657949</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>21</v>
       </c>
@@ -2148,40 +2221,40 @@
         <v>21</v>
       </c>
       <c r="G23">
-        <v>50</v>
-      </c>
-      <c r="H23">
+        <v>43</v>
+      </c>
+      <c r="H23" s="20">
         <v>-153.70000000000002</v>
       </c>
-      <c r="L23" s="2" t="s">
+      <c r="L23" t="s">
         <v>27</v>
       </c>
-      <c r="M23" s="2">
+      <c r="M23">
         <v>6.3260366803859949</v>
       </c>
-      <c r="N23" s="2">
+      <c r="N23">
         <v>0.35812825526203934</v>
       </c>
-      <c r="O23" s="2">
+      <c r="O23">
         <v>17.664165246490501</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="18">
         <v>2.5567165519171674E-19</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23">
         <v>5.5997189143074566</v>
       </c>
-      <c r="R23" s="2">
+      <c r="R23">
         <v>7.0523544464645331</v>
       </c>
-      <c r="S23" s="2">
+      <c r="S23">
         <v>5.5997189143074566</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23">
         <v>7.0523544464645331</v>
       </c>
     </row>
-    <row r="24" spans="2:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24">
         <v>22</v>
       </c>
@@ -2198,40 +2271,40 @@
         <v>45</v>
       </c>
       <c r="G24">
-        <v>-3</v>
-      </c>
-      <c r="H24">
+        <v>-19</v>
+      </c>
+      <c r="H24" s="20">
         <v>-65.099999999999994</v>
       </c>
-      <c r="L24" s="3" t="s">
+      <c r="L24" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="M24" s="3">
+      <c r="M24" s="16">
         <v>11.428941121294507</v>
       </c>
-      <c r="N24" s="3">
+      <c r="N24" s="2">
         <v>0.77649442804417779</v>
       </c>
-      <c r="O24" s="3">
+      <c r="O24" s="2">
         <v>14.718638934836337</v>
       </c>
-      <c r="P24" s="3">
+      <c r="P24" s="17">
         <v>8.3317032495549637E-17</v>
       </c>
-      <c r="Q24" s="3">
+      <c r="Q24" s="2">
         <v>9.8541374299833624</v>
       </c>
-      <c r="R24" s="3">
+      <c r="R24" s="2">
         <v>13.003744812605651</v>
       </c>
-      <c r="S24" s="3">
+      <c r="S24" s="2">
         <v>9.8541374299833624</v>
       </c>
-      <c r="T24" s="3">
+      <c r="T24" s="2">
         <v>13.003744812605651</v>
       </c>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B25">
         <v>23</v>
       </c>
@@ -2248,13 +2321,13 @@
         <v>20</v>
       </c>
       <c r="G25">
-        <v>-14</v>
-      </c>
-      <c r="H25">
+        <v>-60</v>
+      </c>
+      <c r="H25" s="20">
         <v>-190.60000000000002</v>
       </c>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B26">
         <v>24</v>
       </c>
@@ -2271,13 +2344,13 @@
         <v>11</v>
       </c>
       <c r="G26">
-        <v>71</v>
-      </c>
-      <c r="H26">
+        <v>-20</v>
+      </c>
+      <c r="H26" s="20">
         <v>0.80000000000001137</v>
       </c>
     </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:22" ht="18" x14ac:dyDescent="0.35">
       <c r="B27">
         <v>25</v>
       </c>
@@ -2294,13 +2367,16 @@
         <v>18</v>
       </c>
       <c r="G27">
+        <v>-70</v>
+      </c>
+      <c r="H27" s="20">
+        <v>154.69999999999999</v>
+      </c>
+      <c r="L27" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="H27">
-        <v>154.69999999999999</v>
-      </c>
-    </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.45">
+    </row>
+    <row r="28" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B28">
         <v>26</v>
       </c>
@@ -2317,13 +2393,16 @@
         <v>30</v>
       </c>
       <c r="G28">
-        <v>-20</v>
-      </c>
-      <c r="H28">
+        <v>-83</v>
+      </c>
+      <c r="H28" s="20">
         <v>-19</v>
       </c>
-    </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L28" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29">
         <v>27</v>
       </c>
@@ -2340,13 +2419,13 @@
         <v>23</v>
       </c>
       <c r="G29">
-        <v>38</v>
-      </c>
-      <c r="H29">
+        <v>95</v>
+      </c>
+      <c r="H29" s="20">
         <v>57.599999999999994</v>
       </c>
     </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B30">
         <v>28</v>
       </c>
@@ -2363,16 +2442,19 @@
         <v>24</v>
       </c>
       <c r="G30">
-        <v>75</v>
-      </c>
-      <c r="H30">
+        <v>-24</v>
+      </c>
+      <c r="H30" s="20">
         <v>-145.89999999999998</v>
       </c>
-      <c r="L30" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="2:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="L30" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="M30" s="10"/>
+      <c r="U30" s="6"/>
+      <c r="V30" s="6"/>
+    </row>
+    <row r="31" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B31">
         <v>29</v>
       </c>
@@ -2389,13 +2471,21 @@
         <v>36</v>
       </c>
       <c r="G31">
-        <v>42</v>
-      </c>
-      <c r="H31">
+        <v>28</v>
+      </c>
+      <c r="H31" s="20">
         <v>-147.50000000000003</v>
       </c>
-    </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L31" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M31" s="7">
+        <v>0.96863558329428057</v>
+      </c>
+      <c r="U31" s="6"/>
+      <c r="V31" s="6"/>
+    </row>
+    <row r="32" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B32">
         <v>30</v>
       </c>
@@ -2412,17 +2502,21 @@
         <v>18</v>
       </c>
       <c r="G32">
-        <v>25</v>
-      </c>
-      <c r="H32">
+        <v>60</v>
+      </c>
+      <c r="H32" s="20">
         <v>85</v>
       </c>
-      <c r="L32" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="M32" s="5"/>
-    </row>
-    <row r="33" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L32" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M32" s="7">
+        <v>0.93825489322385125</v>
+      </c>
+      <c r="U32" s="6"/>
+      <c r="V32" s="6"/>
+    </row>
+    <row r="33" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B33">
         <v>31</v>
       </c>
@@ -2439,19 +2533,21 @@
         <v>36</v>
       </c>
       <c r="G33">
-        <v>70</v>
-      </c>
-      <c r="H33">
+        <v>-4</v>
+      </c>
+      <c r="H33" s="20">
         <v>177.60000000000002</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="M33" s="2">
-        <v>0.97059445235772324</v>
-      </c>
-    </row>
-    <row r="34" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L33" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="M33" s="11">
+        <v>0.93119830959229144</v>
+      </c>
+      <c r="U33" s="6"/>
+      <c r="V33" s="6"/>
+    </row>
+    <row r="34" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B34">
         <v>32</v>
       </c>
@@ -2468,19 +2564,21 @@
         <v>18</v>
       </c>
       <c r="G34">
-        <v>8</v>
-      </c>
-      <c r="H34">
+        <v>-73</v>
+      </c>
+      <c r="H34" s="20">
         <v>9.1000000000000227</v>
       </c>
-      <c r="L34" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M34" s="2">
-        <v>0.94205359094758878</v>
-      </c>
-    </row>
-    <row r="35" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L34" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="M34" s="7">
+        <v>27.975426766055136</v>
+      </c>
+      <c r="U34" s="6"/>
+      <c r="V34" s="6"/>
+    </row>
+    <row r="35" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35">
         <v>33</v>
       </c>
@@ -2497,19 +2595,21 @@
         <v>10</v>
       </c>
       <c r="G35">
-        <v>-8</v>
-      </c>
-      <c r="H35">
+        <v>-67</v>
+      </c>
+      <c r="H35" s="20">
         <v>-42.5</v>
       </c>
-      <c r="L35" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="M35" s="2">
-        <v>0.93353206020458712</v>
-      </c>
-    </row>
-    <row r="36" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L35" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="M35" s="8">
+        <v>40</v>
+      </c>
+      <c r="U35" s="6"/>
+      <c r="V35" s="6"/>
+    </row>
+    <row r="36" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B36">
         <v>34</v>
       </c>
@@ -2526,19 +2626,15 @@
         <v>43</v>
       </c>
       <c r="G36">
-        <v>7</v>
-      </c>
-      <c r="H36">
+        <v>-29</v>
+      </c>
+      <c r="H36" s="20">
         <v>-172.8</v>
       </c>
-      <c r="L36" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="M36" s="2">
-        <v>27.496870924200266</v>
-      </c>
-    </row>
-    <row r="37" spans="2:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="U36" s="6"/>
+      <c r="V36" s="6"/>
+    </row>
+    <row r="37" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37">
         <v>35</v>
       </c>
@@ -2555,19 +2651,18 @@
         <v>35</v>
       </c>
       <c r="G37">
-        <v>82</v>
-      </c>
-      <c r="H37">
+        <v>-37</v>
+      </c>
+      <c r="H37" s="20">
         <v>-123.59999999999998</v>
       </c>
-      <c r="L37" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M37" s="3">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="38" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L37" t="s">
+        <v>8</v>
+      </c>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6"/>
+    </row>
+    <row r="38" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B38">
         <v>36</v>
       </c>
@@ -2584,13 +2679,31 @@
         <v>46</v>
       </c>
       <c r="G38">
-        <v>-20</v>
-      </c>
-      <c r="H38">
+        <v>20</v>
+      </c>
+      <c r="H38" s="20">
         <v>28.799999999999983</v>
       </c>
-    </row>
-    <row r="39" spans="2:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="L38" s="9"/>
+      <c r="M38" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="N38" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="O38" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="P38" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q38" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="U38" s="6"/>
+      <c r="V38" s="6"/>
+    </row>
+    <row r="39" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B39">
         <v>37</v>
       </c>
@@ -2607,16 +2720,33 @@
         <v>22</v>
       </c>
       <c r="G39">
-        <v>35</v>
-      </c>
-      <c r="H39">
+        <v>-9</v>
+      </c>
+      <c r="H39" s="20">
         <v>62.5</v>
       </c>
-      <c r="L39" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="40" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L39" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="M39" s="7">
+        <v>4</v>
+      </c>
+      <c r="N39" s="7">
+        <v>416236.13215399813</v>
+      </c>
+      <c r="O39" s="7">
+        <v>104059.03303849953</v>
+      </c>
+      <c r="P39" s="7">
+        <v>132.96163444128976</v>
+      </c>
+      <c r="Q39" s="7">
+        <v>1.1928319369407781E-20</v>
+      </c>
+      <c r="U39" s="6"/>
+      <c r="V39" s="6"/>
+    </row>
+    <row r="40" spans="2:22" x14ac:dyDescent="0.3">
       <c r="B40">
         <v>38</v>
       </c>
@@ -2633,29 +2763,29 @@
         <v>22</v>
       </c>
       <c r="G40">
-        <v>81</v>
-      </c>
-      <c r="H40">
+        <v>43</v>
+      </c>
+      <c r="H40" s="20">
         <v>-29.899999999999977</v>
       </c>
-      <c r="L40" s="4"/>
-      <c r="M40" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="N40" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="O40" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="P40" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q40" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="41" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L40" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="M40" s="7">
+        <v>35</v>
+      </c>
+      <c r="N40" s="7">
+        <v>27391.857596001995</v>
+      </c>
+      <c r="O40" s="7">
+        <v>782.62450274291416</v>
+      </c>
+      <c r="P40" s="7"/>
+      <c r="Q40" s="7"/>
+      <c r="U40" s="6"/>
+      <c r="V40" s="6"/>
+    </row>
+    <row r="41" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41">
         <v>39</v>
       </c>
@@ -2672,31 +2802,27 @@
         <v>15</v>
       </c>
       <c r="G41">
-        <v>-4</v>
-      </c>
-      <c r="H41">
+        <v>-8</v>
+      </c>
+      <c r="H41" s="20">
         <v>-113.49999999999997</v>
       </c>
-      <c r="L41" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="M41" s="2">
-        <v>5</v>
-      </c>
-      <c r="N41" s="2">
-        <v>417921.34078884771</v>
-      </c>
-      <c r="O41" s="2">
-        <v>83584.268157769548</v>
-      </c>
-      <c r="P41" s="2">
-        <v>110.54980840399529</v>
-      </c>
-      <c r="Q41" s="2">
-        <v>5.0459699910373937E-20</v>
-      </c>
-    </row>
-    <row r="42" spans="2:20" x14ac:dyDescent="0.45">
+      <c r="L41" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="M41" s="8">
+        <v>39</v>
+      </c>
+      <c r="N41" s="8">
+        <v>443627.98975000012</v>
+      </c>
+      <c r="O41" s="8"/>
+      <c r="P41" s="8"/>
+      <c r="Q41" s="8"/>
+      <c r="U41" s="6"/>
+      <c r="V41" s="6"/>
+    </row>
+    <row r="42" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42">
         <v>40</v>
       </c>
@@ -2713,240 +2839,545 @@
         <v>14</v>
       </c>
       <c r="G42">
+        <v>83</v>
+      </c>
+      <c r="H42" s="20">
+        <v>82.399999999999977</v>
+      </c>
+      <c r="U42" s="6"/>
+      <c r="V42" s="6"/>
+    </row>
+    <row r="43" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="L43" s="9"/>
+      <c r="M43" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N43" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="O43" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="P43" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q43" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="R43" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="S43" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="T43" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="U43" s="6"/>
+      <c r="V43" s="6"/>
+    </row>
+    <row r="44" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="L44" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="M44" s="7">
+        <v>-153.35559836468815</v>
+      </c>
+      <c r="N44" s="7">
+        <v>22.313391092345196</v>
+      </c>
+      <c r="O44" s="7">
+        <v>-6.8728055601238545</v>
+      </c>
+      <c r="P44" s="7">
+        <v>5.5787313752953851E-8</v>
+      </c>
+      <c r="Q44" s="7">
+        <v>-198.65419052740873</v>
+      </c>
+      <c r="R44" s="7">
+        <v>-108.05700620196757</v>
+      </c>
+      <c r="S44" s="7">
+        <v>-198.65419052740873</v>
+      </c>
+      <c r="T44" s="7">
+        <v>-108.05700620196757</v>
+      </c>
+      <c r="U44" s="6"/>
+      <c r="V44" s="6"/>
+    </row>
+    <row r="45" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="L45" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H42">
-        <v>82.399999999999977</v>
-      </c>
-      <c r="L42" s="2" t="s">
+      <c r="M45" s="7">
+        <v>-3.4796531458630033</v>
+      </c>
+      <c r="N45" s="7">
+        <v>0.22927932400182721</v>
+      </c>
+      <c r="O45" s="7">
+        <v>-15.176480308513439</v>
+      </c>
+      <c r="P45" s="7">
+        <v>5.7651808900406986E-17</v>
+      </c>
+      <c r="Q45" s="7">
+        <v>-3.9451149193029922</v>
+      </c>
+      <c r="R45" s="7">
+        <v>-3.0141913724230145</v>
+      </c>
+      <c r="S45" s="7">
+        <v>-3.9451149193029922</v>
+      </c>
+      <c r="T45" s="7">
+        <v>-3.0141913724230145</v>
+      </c>
+      <c r="U45" s="6"/>
+      <c r="V45" s="6"/>
+    </row>
+    <row r="46" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="L46" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="M46" s="7">
+        <v>6.3073152440645712</v>
+      </c>
+      <c r="N46" s="7">
+        <v>0.36349366606800393</v>
+      </c>
+      <c r="O46" s="7">
+        <v>17.351926134758486</v>
+      </c>
+      <c r="P46" s="7">
+        <v>9.0690618861468427E-19</v>
+      </c>
+      <c r="Q46" s="7">
+        <v>5.5693838707111336</v>
+      </c>
+      <c r="R46" s="7">
+        <v>7.0452466174180088</v>
+      </c>
+      <c r="S46" s="7">
+        <v>5.5693838707111336</v>
+      </c>
+      <c r="T46" s="7">
+        <v>7.0452466174180088</v>
+      </c>
+      <c r="U46" s="6"/>
+      <c r="V46" s="6"/>
+    </row>
+    <row r="47" spans="2:22" x14ac:dyDescent="0.3">
+      <c r="L47" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M47" s="7">
+        <v>11.546974317916742</v>
+      </c>
+      <c r="N47" s="7">
+        <v>0.81551612655375483</v>
+      </c>
+      <c r="O47" s="7">
+        <v>14.159099914691414</v>
+      </c>
+      <c r="P47" s="7">
+        <v>4.6958110639733952E-16</v>
+      </c>
+      <c r="Q47" s="7">
+        <v>9.8913885637839538</v>
+      </c>
+      <c r="R47" s="7">
+        <v>13.202560072049531</v>
+      </c>
+      <c r="S47" s="7">
+        <v>9.8913885637839538</v>
+      </c>
+      <c r="T47" s="7">
+        <v>13.202560072049531</v>
+      </c>
+      <c r="U47" s="6"/>
+      <c r="V47" s="6"/>
+    </row>
+    <row r="48" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L48" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="M48" s="8">
+        <v>0.19769153345241794</v>
+      </c>
+      <c r="N48" s="8">
+        <v>0.37381185659844346</v>
+      </c>
+      <c r="O48" s="8">
+        <v>0.52885303117814786</v>
+      </c>
+      <c r="P48" s="13">
+        <v>0.60024549371244085</v>
+      </c>
+      <c r="Q48" s="8">
+        <v>-0.56118688030206265</v>
+      </c>
+      <c r="R48" s="8">
+        <v>0.95656994720689859</v>
+      </c>
+      <c r="S48" s="8">
+        <v>-0.56118688030206265</v>
+      </c>
+      <c r="T48" s="8">
+        <v>0.95656994720689859</v>
+      </c>
+      <c r="U48" s="6"/>
+      <c r="V48" s="6"/>
+    </row>
+    <row r="49" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="U49" s="6"/>
+      <c r="V49" s="6"/>
+    </row>
+    <row r="50" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="U50" s="6"/>
+      <c r="V50" s="6"/>
+    </row>
+    <row r="51" spans="12:22" ht="18" x14ac:dyDescent="0.35">
+      <c r="L51" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="U51" s="6"/>
+      <c r="V51" s="6"/>
+    </row>
+    <row r="52" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L52" t="s">
+        <v>1</v>
+      </c>
+      <c r="U52" s="6"/>
+      <c r="V52" s="6"/>
+    </row>
+    <row r="53" spans="12:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="U53" s="6"/>
+      <c r="V53" s="6"/>
+    </row>
+    <row r="54" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L54" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="M54" s="10"/>
+      <c r="U54" s="6"/>
+      <c r="V54" s="6"/>
+    </row>
+    <row r="55" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L55" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="M55" s="7">
+        <v>0.96869680119410473</v>
+      </c>
+    </row>
+    <row r="56" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L56" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M56" s="7">
+        <v>0.93837349264369085</v>
+      </c>
+    </row>
+    <row r="57" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L57" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="M57" s="11">
+        <v>0.92931077097364534</v>
+      </c>
+    </row>
+    <row r="58" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L58" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="M58" s="7">
+        <v>28.356575943318806</v>
+      </c>
+    </row>
+    <row r="59" spans="12:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L59" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="M59" s="8">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61" spans="12:22" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L61" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L62" s="9"/>
+      <c r="M62" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="N62" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="O62" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="P62" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q62" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="63" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L63" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="M63" s="7">
+        <v>5</v>
+      </c>
+      <c r="N63" s="7">
+        <v>416288.74617620709</v>
+      </c>
+      <c r="O63" s="7">
+        <v>83257.749235241412</v>
+      </c>
+      <c r="P63" s="7">
+        <v>103.5421286019681</v>
+      </c>
+      <c r="Q63" s="7">
+        <v>1.4293634690104051E-19</v>
+      </c>
+    </row>
+    <row r="64" spans="12:22" x14ac:dyDescent="0.3">
+      <c r="L64" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="M42" s="2">
+      <c r="M64" s="7">
         <v>34</v>
       </c>
-      <c r="N42" s="2">
-        <v>25706.648961152423</v>
-      </c>
-      <c r="O42" s="2">
-        <v>756.07791062213005</v>
-      </c>
-      <c r="P42" s="2"/>
-      <c r="Q42" s="2"/>
-    </row>
-    <row r="43" spans="2:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="L43" s="3" t="s">
+      <c r="N64" s="7">
+        <v>27339.243573793032</v>
+      </c>
+      <c r="O64" s="7">
+        <v>804.09539922920681</v>
+      </c>
+      <c r="P64" s="7"/>
+      <c r="Q64" s="7"/>
+    </row>
+    <row r="65" spans="12:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L65" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M43" s="3">
+      <c r="M65" s="8">
         <v>39</v>
       </c>
-      <c r="N43" s="3">
+      <c r="N65" s="8">
         <v>443627.98975000012</v>
       </c>
-      <c r="O43" s="3"/>
-      <c r="P43" s="3"/>
-      <c r="Q43" s="3"/>
-    </row>
-    <row r="44" spans="2:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="45" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="L45" s="4"/>
-      <c r="M45" s="4" t="s">
+      <c r="O65" s="8"/>
+      <c r="P65" s="8"/>
+      <c r="Q65" s="8"/>
+    </row>
+    <row r="66" spans="12:20" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="67" spans="12:20" x14ac:dyDescent="0.3">
+      <c r="L67" s="9"/>
+      <c r="M67" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="N45" s="4" t="s">
+      <c r="N67" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="O45" s="4" t="s">
+      <c r="O67" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="P45" s="4" t="s">
+      <c r="P67" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="Q45" s="4" t="s">
+      <c r="Q67" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="R45" s="4" t="s">
+      <c r="R67" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="S45" s="4" t="s">
+      <c r="S67" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="T45" s="4" t="s">
+      <c r="T67" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="L46" s="2" t="s">
+    <row r="68" spans="12:20" x14ac:dyDescent="0.3">
+      <c r="L68" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="M46" s="2">
-        <v>-163.53527701928843</v>
-      </c>
-      <c r="N46" s="2">
-        <v>22.967180895548086</v>
-      </c>
-      <c r="O46" s="2">
-        <v>-7.1203896448165214</v>
-      </c>
-      <c r="P46" s="2">
-        <v>3.1463751906525252E-8</v>
-      </c>
-      <c r="Q46" s="2">
-        <v>-210.21020428877284</v>
-      </c>
-      <c r="R46" s="2">
-        <v>-116.86034974980402</v>
-      </c>
-      <c r="S46" s="2">
-        <v>-210.21020428877284</v>
-      </c>
-      <c r="T46" s="2">
-        <v>-116.86034974980402</v>
-      </c>
-    </row>
-    <row r="47" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="L47" s="2" t="s">
+      <c r="M68" s="7">
+        <v>-154.48971484218077</v>
+      </c>
+      <c r="N68" s="7">
+        <v>23.047860916573335</v>
+      </c>
+      <c r="O68" s="7">
+        <v>-6.7029957965031706</v>
+      </c>
+      <c r="P68" s="7">
+        <v>1.0682068870911217E-7</v>
+      </c>
+      <c r="Q68" s="7">
+        <v>-201.32860364140538</v>
+      </c>
+      <c r="R68" s="7">
+        <v>-107.65082604295617</v>
+      </c>
+      <c r="S68" s="7">
+        <v>-201.32860364140538</v>
+      </c>
+      <c r="T68" s="7">
+        <v>-107.65082604295617</v>
+      </c>
+    </row>
+    <row r="69" spans="12:20" x14ac:dyDescent="0.3">
+      <c r="L69" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="M47" s="2">
-        <v>-3.4534635226024126</v>
-      </c>
-      <c r="N47" s="2">
-        <v>0.22603893652062002</v>
-      </c>
-      <c r="O47" s="2">
-        <v>-15.278179838221705</v>
-      </c>
-      <c r="P47" s="2">
-        <v>8.581501965141885E-17</v>
-      </c>
-      <c r="Q47" s="2">
-        <v>-3.9128299102384592</v>
-      </c>
-      <c r="R47" s="2">
-        <v>-2.9940971349663661</v>
-      </c>
-      <c r="S47" s="2">
-        <v>-3.9128299102384592</v>
-      </c>
-      <c r="T47" s="2">
-        <v>-2.9940971349663661</v>
-      </c>
-    </row>
-    <row r="48" spans="2:20" x14ac:dyDescent="0.45">
-      <c r="L48" s="2" t="s">
+      <c r="M69" s="7">
+        <v>-3.4747136835597541</v>
+      </c>
+      <c r="N69" s="7">
+        <v>0.2332039637141694</v>
+      </c>
+      <c r="O69" s="7">
+        <v>-14.899891186320481</v>
+      </c>
+      <c r="P69" s="7">
+        <v>1.8071248973967142E-16</v>
+      </c>
+      <c r="Q69" s="7">
+        <v>-3.9486411583690035</v>
+      </c>
+      <c r="R69" s="7">
+        <v>-3.0007862087505046</v>
+      </c>
+      <c r="S69" s="7">
+        <v>-3.9486411583690035</v>
+      </c>
+      <c r="T69" s="7">
+        <v>-3.0007862087505046</v>
+      </c>
+    </row>
+    <row r="70" spans="12:20" x14ac:dyDescent="0.3">
+      <c r="L70" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="M48" s="2">
-        <v>6.2781874454700315</v>
-      </c>
-      <c r="N48" s="2">
-        <v>0.35780795526858672</v>
-      </c>
-      <c r="O48" s="2">
-        <v>17.546248910976118</v>
-      </c>
-      <c r="P48" s="2">
-        <v>1.2999241098274708E-18</v>
-      </c>
-      <c r="Q48" s="2">
-        <v>5.551034192985246</v>
-      </c>
-      <c r="R48" s="2">
-        <v>7.005340697954817</v>
-      </c>
-      <c r="S48" s="2">
-        <v>5.551034192985246</v>
-      </c>
-      <c r="T48" s="2">
-        <v>7.005340697954817</v>
-      </c>
-    </row>
-    <row r="49" spans="12:20" x14ac:dyDescent="0.45">
-      <c r="L49" s="2" t="s">
+      <c r="M70" s="7">
+        <v>6.3316947614106516</v>
+      </c>
+      <c r="N70" s="7">
+        <v>0.38057333399317084</v>
+      </c>
+      <c r="O70" s="7">
+        <v>16.637252786408492</v>
+      </c>
+      <c r="P70" s="7">
+        <v>6.6024150997683889E-18</v>
+      </c>
+      <c r="Q70" s="7">
+        <v>5.558276693010292</v>
+      </c>
+      <c r="R70" s="7">
+        <v>7.1051128298110111</v>
+      </c>
+      <c r="S70" s="7">
+        <v>5.558276693010292</v>
+      </c>
+      <c r="T70" s="7">
+        <v>7.1051128298110111</v>
+      </c>
+    </row>
+    <row r="71" spans="12:20" x14ac:dyDescent="0.3">
+      <c r="L71" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="M49" s="2">
-        <v>11.517572560741451</v>
-      </c>
-      <c r="N49" s="2">
-        <v>0.80180756274379084</v>
-      </c>
-      <c r="O49" s="2">
-        <v>14.364509760082882</v>
-      </c>
-      <c r="P49" s="2">
-        <v>5.3123569690149874E-16</v>
-      </c>
-      <c r="Q49" s="2">
-        <v>9.8881035438259595</v>
-      </c>
-      <c r="R49" s="2">
-        <v>13.147041577656942</v>
-      </c>
-      <c r="S49" s="2">
-        <v>9.8881035438259595</v>
-      </c>
-      <c r="T49" s="2">
-        <v>13.147041577656942</v>
-      </c>
-    </row>
-    <row r="50" spans="12:20" x14ac:dyDescent="0.45">
-      <c r="L50" s="2" t="s">
+      <c r="M71" s="7">
+        <v>11.523409594527093</v>
+      </c>
+      <c r="N71" s="7">
+        <v>0.83174446190688323</v>
+      </c>
+      <c r="O71" s="7">
+        <v>13.854507150078483</v>
+      </c>
+      <c r="P71" s="7">
+        <v>1.525194475312969E-15</v>
+      </c>
+      <c r="Q71" s="7">
+        <v>9.8331014786614084</v>
+      </c>
+      <c r="R71" s="7">
+        <v>13.213717710392778</v>
+      </c>
+      <c r="S71" s="7">
+        <v>9.8331014786614084</v>
+      </c>
+      <c r="T71" s="7">
+        <v>13.213717710392778</v>
+      </c>
+    </row>
+    <row r="72" spans="12:20" x14ac:dyDescent="0.3">
+      <c r="L72" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="M50" s="2">
-        <v>0.29973713937674529</v>
-      </c>
-      <c r="N50" s="2">
-        <v>0.37372111756563919</v>
-      </c>
-      <c r="O50" s="2">
-        <v>0.8020342584041974</v>
-      </c>
-      <c r="P50" s="2">
-        <v>0.42810355403979372</v>
-      </c>
-      <c r="Q50" s="2">
-        <v>-0.45975554981210676</v>
-      </c>
-      <c r="R50" s="2">
-        <v>1.0592298285655972</v>
-      </c>
-      <c r="S50" s="2">
-        <v>-0.45975554981210676</v>
-      </c>
-      <c r="T50" s="2">
-        <v>1.0592298285655972</v>
-      </c>
-    </row>
-    <row r="51" spans="12:20" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="L51" s="3" t="s">
+      <c r="M72" s="7">
+        <v>0.20579931933704809</v>
+      </c>
+      <c r="N72" s="7">
+        <v>0.38022823399340661</v>
+      </c>
+      <c r="O72" s="7">
+        <v>0.54125207161921796</v>
+      </c>
+      <c r="P72" s="15">
+        <v>0.59186296124984317</v>
+      </c>
+      <c r="Q72" s="7">
+        <v>-0.56691742148362534</v>
+      </c>
+      <c r="R72" s="7">
+        <v>0.97851606015772152</v>
+      </c>
+      <c r="S72" s="7">
+        <v>-0.56691742148362534</v>
+      </c>
+      <c r="T72" s="7">
+        <v>0.97851606015772152</v>
+      </c>
+    </row>
+    <row r="73" spans="12:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L73" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="M51" s="3">
-        <v>0.20514658461374533</v>
-      </c>
-      <c r="N51" s="3">
-        <v>0.13741075572673345</v>
-      </c>
-      <c r="O51" s="3">
-        <v>1.4929441551265246</v>
-      </c>
-      <c r="P51" s="3">
-        <v>0.1446741907906621</v>
-      </c>
-      <c r="Q51" s="3">
-        <v>-7.4105669233107047E-2</v>
-      </c>
-      <c r="R51" s="3">
-        <v>0.48439883846059772</v>
-      </c>
-      <c r="S51" s="3">
-        <v>-7.4105669233107047E-2</v>
-      </c>
-      <c r="T51" s="3">
-        <v>0.48439883846059772</v>
+      <c r="M73" s="8">
+        <v>-2.4297348586997593E-2</v>
+      </c>
+      <c r="N73" s="8">
+        <v>9.4986507825756003E-2</v>
+      </c>
+      <c r="O73" s="8">
+        <v>-0.25579789322888719</v>
+      </c>
+      <c r="P73" s="13">
+        <v>0.79964817645098163</v>
+      </c>
+      <c r="Q73" s="8">
+        <v>-0.21733315757515478</v>
+      </c>
+      <c r="R73" s="8">
+        <v>0.16873846040115961</v>
+      </c>
+      <c r="S73" s="8">
+        <v>-0.21733315757515478</v>
+      </c>
+      <c r="T73" s="8">
+        <v>0.16873846040115961</v>
       </c>
     </row>
   </sheetData>

</xml_diff>